<commit_message>
Adiciona planilhas XLSX formatadas para dados abertos
</commit_message>
<xml_diff>
--- a/dados/excel/genero_geral.xlsx
+++ b/dados/excel/genero_geral.xlsx
@@ -7,18 +7,25 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metadados" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Metadados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dados" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cobertura gênero" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dados'!$A$1:$H$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,14 +35,37 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="000D2B4E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +74,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00003A70"/>
-        <bgColor rgb="00003A70"/>
+        <fgColor rgb="000D2B4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -58,26 +92,69 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color rgb="004A90D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8DEE6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D8DEE6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D8DEE6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D8DEE6"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,188 +520,293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GÊNERO</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>REGISTROS</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>MATRÍCULAS ÚNICAS</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>FOLHA BRUTA (R$)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>FOLHA MÉDIA (R$)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>FOLHA MEDIANA (R$)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>PERCENTUAL_MATRICULAS</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>PARTICIPAÇÃO NA FOLHA (%)</t>
+          <t>Gênero (geral)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>feminino</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>647640</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>20640</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>4054649639.44</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>6260.653510345253</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>4583.34</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>78.25</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>69.23</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>masculino</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>191623</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>5426</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>1719022989.33</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>8970.859392296332</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>6455.84</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>20.57</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>29.35</t>
+          <t>Fonte: Portal da Transparência de Sorocaba · Organizado pelo Observatório Social do Brasil — Sorocaba · Licença CC-BY 4.0</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>indefinido</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>11254</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>312</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>82983874.94</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>7373.722671050293</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>5520.74</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>1.18</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>1.42</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Para que serve</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Quantos F e M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Informações técnicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Arquivo</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>genero_geral.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distribuição geral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Linhas</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Colunas</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Separador</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ponto e vírgula</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Codificação</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>utf-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Gerado em</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026 19:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Dicionário de colunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Coluna</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Formato no Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>﻿genero_inferido</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Número decimal (#,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>num_registros</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Número decimal (#,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>num_matriculas</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Número decimal (#,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>folha_total</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>moeda</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Moeda (R$ #,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>folha_media</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>moeda</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Moeda (R$ #,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>folha_mediana</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>moeda</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Moeda (R$ #,##0,00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>percentual_matriculas</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Percentual (0,0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>percentual_folha</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Percentual (0,0%)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -635,83 +817,229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>﻿genero_inferido</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>num_registros</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>num_matriculas</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>folha_total</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>folha_media</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>folha_mediana</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>percentual_matriculas</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>percentual_folha</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>feminino</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>647640</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>20640</v>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>4054649639.44</v>
+      </c>
+      <c r="E2" s="10" t="n">
+        <v>6260.653510345253</v>
+      </c>
+      <c r="F2" s="10" t="n">
+        <v>4583.34</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>69.23</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n">
+        <v>191623</v>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>5426</v>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>1719022989.33</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>8970.859392296332</v>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>6455.84</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>29.35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>indefinido</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>11254</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>312</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>82983874.94</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>7373.722671050293</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>5520.74</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CAMPO</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>FONTE</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Portal da Transparência de Sorocaba</t>
+          <t>Cobertura da análise de gênero</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>https://transparencia.sorocaba.sp.gov.br</t>
-        </is>
+          <t>Matrículas totais</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="n">
+        <v>26378</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>PERÍODO</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>2022-01 a 2026-08</t>
-        </is>
+          <t>Classificadas F/M</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>26066</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>LICENÇA</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>CC-BY 4.0 — Observatório Social do Brasil — Sorocaba</t>
-        </is>
+          <t>Indefinidas</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>312</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>GERADO EM</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-23 18:50</t>
-        </is>
+          <t>Feminino</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>20640</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Masculino</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>5426</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Cobertura</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>98.81999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>